<commit_message>
Updates to correct over zealous trimming of packets pre-launch and post-landing
</commit_message>
<xml_diff>
--- a/www/flightdata/xlsx/eoss-387.xlsx
+++ b/www/flightdata/xlsx/eoss-387.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1448" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="540">
   <si>
     <t>flight</t>
   </si>
@@ -147,7 +147,7 @@
     <t>344</t>
   </si>
   <si>
-    <t>1hrs 36mins 7secs</t>
+    <t>1hrs 48mins 37secs</t>
   </si>
   <si>
     <t>flightid</t>
@@ -1332,6 +1332,12 @@
     <t>/161915h3924.91N/10228.66WO156/011/A=005090 41T8467P EOSS Balloon</t>
   </si>
   <si>
+    <t>/161945h3924.84N/10228.63WO140/007/A=004606 46T8622P EOSS Balloon</t>
+  </si>
+  <si>
+    <t>/163145h3924.76N/10228.59WO170/000/A=004206 138T8762P EOSS Balloon</t>
+  </si>
+  <si>
     <t>KC0D-2&gt;APZEOS,EOSS,WIDE2-1,qAO,N0JD-10:/153645h3949.83N/10318.10WO186/016/A=080016 13T261P EOSS Balloon</t>
   </si>
   <si>
@@ -1621,6 +1627,12 @@
   </si>
   <si>
     <t>KC0D-2&gt;APZEOS,EOSS*,WIDE2-1,qAO,W9CN-9:/161915h3924.91N/10228.66WO156/011/A=005090 41T8467P EOSS Balloon</t>
+  </si>
+  <si>
+    <t>KC0D-2&gt;APZEOS,EOSS*,WIDE2-1,qAO,W9CN-9:/161945h3924.84N/10228.63WO140/007/A=004606 46T8622P EOSS Balloon</t>
+  </si>
+  <si>
+    <t>KC0D-2&gt;APZEOS,EOSS,WIDE2-1,qAO,KE0UWC-9:/163145h3924.76N/10228.59WO170/000/A=004206 138T8762P EOSS Balloon</t>
   </si>
   <si>
     <t>n/a</t>
@@ -2127,19 +2139,19 @@
         <v>27272.59</v>
       </c>
       <c r="I2">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="J2" t="s">
         <v>43</v>
       </c>
       <c r="K2">
-        <v>5767</v>
+        <v>6517</v>
       </c>
       <c r="L2">
-        <v>101.55</v>
+        <v>101.7</v>
       </c>
       <c r="M2">
-        <v>163.43</v>
+        <v>163.66</v>
       </c>
       <c r="N2">
         <v>9.630000000000001</v>
@@ -2196,22 +2208,22 @@
         <v>1418.84</v>
       </c>
       <c r="AF2">
-        <v>39.4151666667</v>
+        <v>39.4126666667</v>
       </c>
       <c r="AG2">
-        <v>-102.4776666667</v>
+        <v>-102.4765</v>
       </c>
       <c r="AH2">
-        <v>101.55</v>
+        <v>101.7</v>
       </c>
       <c r="AI2">
-        <v>163.43</v>
+        <v>163.66</v>
       </c>
       <c r="AJ2">
-        <v>5090</v>
+        <v>4206</v>
       </c>
       <c r="AK2">
-        <v>1551.43</v>
+        <v>1281.99</v>
       </c>
     </row>
   </sheetData>
@@ -19272,7 +19284,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AU98"/>
+  <dimension ref="A1:AU100"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:47">
@@ -19450,7 +19462,7 @@
         <v>341</v>
       </c>
       <c r="K2" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="L2">
         <v>186</v>
@@ -19507,19 +19519,19 @@
         <v>-24.03091667</v>
       </c>
       <c r="AD2" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AF2">
         <v>-78.841667</v>
       </c>
       <c r="AL2">
-        <v>-78.84302700000001</v>
+        <v>-78.87849199999999</v>
       </c>
       <c r="AN2">
         <v>-24.030917</v>
       </c>
       <c r="AT2">
-        <v>-24.03134</v>
+        <v>-24.042151</v>
       </c>
     </row>
     <row r="3" spans="1:47">
@@ -19554,7 +19566,7 @@
         <v>342</v>
       </c>
       <c r="K3" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="L3">
         <v>163</v>
@@ -19611,7 +19623,7 @@
         <v>-25.68466667</v>
       </c>
       <c r="AD3" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE3">
         <v>-0.180833</v>
@@ -19629,7 +19641,7 @@
         <v>-0.707107</v>
       </c>
       <c r="AL3">
-        <v>-84.22279</v>
+        <v>-84.035376</v>
       </c>
       <c r="AM3">
         <v>-0.055125</v>
@@ -19647,7 +19659,7 @@
         <v>-0.707106</v>
       </c>
       <c r="AT3">
-        <v>-25.671228</v>
+        <v>-25.614101</v>
       </c>
     </row>
     <row r="4" spans="1:47">
@@ -19682,7 +19694,7 @@
         <v>343</v>
       </c>
       <c r="K4" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="L4">
         <v>136</v>
@@ -19739,7 +19751,7 @@
         <v>-25.17633333</v>
       </c>
       <c r="AD4" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE4">
         <v>0.055556</v>
@@ -19763,7 +19775,7 @@
         <v>0.707105</v>
       </c>
       <c r="AL4">
-        <v>-82.979866</v>
+        <v>-83.263727</v>
       </c>
       <c r="AM4">
         <v>0.016944</v>
@@ -19787,7 +19799,7 @@
         <v>0.707104</v>
       </c>
       <c r="AT4">
-        <v>-25.292287</v>
+        <v>-25.378812</v>
       </c>
     </row>
     <row r="5" spans="1:47">
@@ -19822,7 +19834,7 @@
         <v>344</v>
       </c>
       <c r="K5" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="L5">
         <v>140</v>
@@ -19879,7 +19891,7 @@
         <v>-24.14033333</v>
       </c>
       <c r="AD5" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE5">
         <v>0.113333</v>
@@ -19903,7 +19915,7 @@
         <v>0.7526929999999999</v>
       </c>
       <c r="AL5">
-        <v>-77.95558</v>
+        <v>-77.985331</v>
       </c>
       <c r="AM5">
         <v>0.034533</v>
@@ -19927,7 +19939,7 @@
         <v>0.752484</v>
       </c>
       <c r="AT5">
-        <v>-23.760869</v>
+        <v>-23.769937</v>
       </c>
     </row>
     <row r="6" spans="1:47">
@@ -19962,7 +19974,7 @@
         <v>345</v>
       </c>
       <c r="K6" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="L6">
         <v>229</v>
@@ -20019,7 +20031,7 @@
         <v>-21.92533333</v>
       </c>
       <c r="AD6" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE6">
         <v>0.242222</v>
@@ -20043,7 +20055,7 @@
         <v>1.042908</v>
       </c>
       <c r="AL6">
-        <v>-73.100436</v>
+        <v>-72.906808</v>
       </c>
       <c r="AM6">
         <v>0.073833</v>
@@ -20067,7 +20079,7 @@
         <v>1.042931</v>
       </c>
       <c r="AT6">
-        <v>-22.281037</v>
+        <v>-22.222017</v>
       </c>
     </row>
     <row r="7" spans="1:47">
@@ -20102,7 +20114,7 @@
         <v>346</v>
       </c>
       <c r="K7" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="L7">
         <v>194</v>
@@ -20159,7 +20171,7 @@
         <v>-20.74666667</v>
       </c>
       <c r="AD7" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE7">
         <v>0.128889</v>
@@ -20183,7 +20195,7 @@
         <v>0.364303</v>
       </c>
       <c r="AL7">
-        <v>-69.150603</v>
+        <v>-68.983672</v>
       </c>
       <c r="AM7">
         <v>0.039289</v>
@@ -20207,7 +20219,7 @@
         <v>0.364349</v>
       </c>
       <c r="AT7">
-        <v>-21.07713</v>
+        <v>-21.026247</v>
       </c>
     </row>
     <row r="8" spans="1:47">
@@ -20242,7 +20254,7 @@
         <v>347</v>
       </c>
       <c r="K8" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="L8">
         <v>70</v>
@@ -20299,7 +20311,7 @@
         <v>-20.452</v>
       </c>
       <c r="AD8" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE8">
         <v>0.032222</v>
@@ -20323,7 +20335,7 @@
         <v>-0.234092</v>
       </c>
       <c r="AL8">
-        <v>-65.675911</v>
+        <v>-65.676137</v>
       </c>
       <c r="AM8">
         <v>0.009821999999999999</v>
@@ -20347,7 +20359,7 @@
         <v>-0.234069</v>
       </c>
       <c r="AT8">
-        <v>-20.018024</v>
+        <v>-20.018093</v>
       </c>
     </row>
     <row r="9" spans="1:47">
@@ -20382,7 +20394,7 @@
         <v>348</v>
       </c>
       <c r="K9" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="L9">
         <v>161</v>
@@ -20439,7 +20451,7 @@
         <v>-19.38533333</v>
       </c>
       <c r="AD9" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE9">
         <v>0.116667</v>
@@ -20463,7 +20475,7 @@
         <v>0.338654</v>
       </c>
       <c r="AL9">
-        <v>-62.347226</v>
+        <v>-62.487933</v>
       </c>
       <c r="AM9">
         <v>0.035556</v>
@@ -20487,7 +20499,7 @@
         <v>0.338533</v>
       </c>
       <c r="AT9">
-        <v>-19.003408</v>
+        <v>-19.046298</v>
       </c>
     </row>
     <row r="10" spans="1:47">
@@ -20522,7 +20534,7 @@
         <v>349</v>
       </c>
       <c r="K10" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="L10">
         <v>41</v>
@@ -20579,7 +20591,7 @@
         <v>-18.01366667</v>
       </c>
       <c r="AD10" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE10">
         <v>0.15</v>
@@ -20603,7 +20615,7 @@
         <v>0.548091</v>
       </c>
       <c r="AL10">
-        <v>-58.989134</v>
+        <v>-59.16611</v>
       </c>
       <c r="AM10">
         <v>0.045722</v>
@@ -20627,7 +20639,7 @@
         <v>0.548109</v>
       </c>
       <c r="AT10">
-        <v>-17.979844</v>
+        <v>-18.033789</v>
       </c>
     </row>
     <row r="11" spans="1:47">
@@ -20662,7 +20674,7 @@
         <v>350</v>
       </c>
       <c r="K11" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="L11">
         <v>84</v>
@@ -20719,7 +20731,7 @@
         <v>-16.36766667</v>
       </c>
       <c r="AD11" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE11">
         <v>0.18</v>
@@ -20743,7 +20755,7 @@
         <v>0.723314</v>
       </c>
       <c r="AL11">
-        <v>-55.702069</v>
+        <v>-55.827605</v>
       </c>
       <c r="AM11">
         <v>0.054867</v>
@@ -20767,7 +20779,7 @@
         <v>0.723357</v>
       </c>
       <c r="AT11">
-        <v>-16.977948</v>
+        <v>-17.016213</v>
       </c>
     </row>
     <row r="12" spans="1:47">
@@ -20802,7 +20814,7 @@
         <v>351</v>
       </c>
       <c r="K12" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="L12">
         <v>179</v>
@@ -20859,7 +20871,7 @@
         <v>-15.88</v>
       </c>
       <c r="AD12" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE12">
         <v>0.053333</v>
@@ -20883,7 +20895,7 @@
         <v>-0.314239</v>
       </c>
       <c r="AL12">
-        <v>-52.405166</v>
+        <v>-52.434269</v>
       </c>
       <c r="AM12">
         <v>0.016256</v>
@@ -20907,7 +20919,7 @@
         <v>-0.314226</v>
       </c>
       <c r="AT12">
-        <v>-15.973065</v>
+        <v>-15.981936</v>
       </c>
     </row>
     <row r="13" spans="1:47">
@@ -20942,7 +20954,7 @@
         <v>352</v>
       </c>
       <c r="K13" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="L13">
         <v>147</v>
@@ -20999,7 +21011,7 @@
         <v>-15.11833333</v>
       </c>
       <c r="AD13" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE13">
         <v>0.083333</v>
@@ -21023,7 +21035,7 @@
         <v>-0.04882</v>
       </c>
       <c r="AL13">
-        <v>-49.314215</v>
+        <v>-49.247092</v>
       </c>
       <c r="AM13">
         <v>0.025389</v>
@@ -21047,7 +21059,7 @@
         <v>-0.049128</v>
       </c>
       <c r="AT13">
-        <v>-15.030942</v>
+        <v>-15.010481</v>
       </c>
     </row>
     <row r="14" spans="1:47">
@@ -21082,7 +21094,7 @@
         <v>353</v>
       </c>
       <c r="K14" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="L14">
         <v>147</v>
@@ -21139,7 +21151,7 @@
         <v>-14.112</v>
       </c>
       <c r="AD14" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE14">
         <v>0.11</v>
@@ -21163,7 +21175,7 @@
         <v>0.189859</v>
       </c>
       <c r="AL14">
-        <v>-46.599457</v>
+        <v>-46.467669</v>
       </c>
       <c r="AM14">
         <v>0.033544</v>
@@ -21187,7 +21199,7 @@
         <v>0.190355</v>
       </c>
       <c r="AT14">
-        <v>-14.203515</v>
+        <v>-14.163344</v>
       </c>
     </row>
     <row r="15" spans="1:47">
@@ -21222,7 +21234,7 @@
         <v>354</v>
       </c>
       <c r="K15" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="L15">
         <v>118</v>
@@ -21279,7 +21291,7 @@
         <v>-13.401</v>
       </c>
       <c r="AD15" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE15">
         <v>0.077778</v>
@@ -21303,7 +21315,7 @@
         <v>-0.117708</v>
       </c>
       <c r="AL15">
-        <v>-44.26307</v>
+        <v>-44.107728</v>
       </c>
       <c r="AM15">
         <v>0.0237</v>
@@ -21327,7 +21339,7 @@
         <v>-0.117916</v>
       </c>
       <c r="AT15">
-        <v>-13.4914</v>
+        <v>-13.44405</v>
       </c>
     </row>
     <row r="16" spans="1:47">
@@ -21362,7 +21374,7 @@
         <v>355</v>
       </c>
       <c r="K16" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="L16">
         <v>105</v>
@@ -21419,7 +21431,7 @@
         <v>-13.10666667</v>
       </c>
       <c r="AD16" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE16">
         <v>0.032222</v>
@@ -21443,7 +21455,7 @@
         <v>-0.551718</v>
       </c>
       <c r="AL16">
-        <v>-42.255893</v>
+        <v>-42.116559</v>
       </c>
       <c r="AM16">
         <v>0.009811</v>
@@ -21467,7 +21479,7 @@
         <v>-0.552</v>
       </c>
       <c r="AT16">
-        <v>-12.879612</v>
+        <v>-12.837141</v>
       </c>
     </row>
     <row r="17" spans="1:46">
@@ -21502,7 +21514,7 @@
         <v>356</v>
       </c>
       <c r="K17" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="L17">
         <v>125</v>
@@ -21559,7 +21571,7 @@
         <v>-12.54733333</v>
       </c>
       <c r="AD17" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE17">
         <v>0.061111</v>
@@ -21583,7 +21595,7 @@
         <v>-0.243181</v>
       </c>
       <c r="AL17">
-        <v>-40.606554</v>
+        <v>-40.513168</v>
       </c>
       <c r="AM17">
         <v>0.018644</v>
@@ -21607,7 +21619,7 @@
         <v>-0.242564</v>
       </c>
       <c r="AT17">
-        <v>-12.37691</v>
+        <v>-12.348445</v>
       </c>
     </row>
     <row r="18" spans="1:46">
@@ -21642,7 +21654,7 @@
         <v>357</v>
       </c>
       <c r="K18" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="L18">
         <v>120</v>
@@ -21699,7 +21711,7 @@
         <v>-12.436</v>
       </c>
       <c r="AD18" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE18">
         <v>0.012222</v>
@@ -21723,7 +21735,7 @@
         <v>-0.731867</v>
       </c>
       <c r="AL18">
-        <v>-39.222181</v>
+        <v>-39.192722</v>
       </c>
       <c r="AM18">
         <v>0.003711</v>
@@ -21747,7 +21759,7 @@
         <v>-0.732297</v>
       </c>
       <c r="AT18">
-        <v>-11.954949</v>
+        <v>-11.94597</v>
       </c>
     </row>
     <row r="19" spans="1:46">
@@ -21782,7 +21794,7 @@
         <v>358</v>
       </c>
       <c r="K19" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="L19">
         <v>102</v>
@@ -21839,7 +21851,7 @@
         <v>-11.88733333</v>
       </c>
       <c r="AD19" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE19">
         <v>0.06</v>
@@ -21863,7 +21875,7 @@
         <v>-0.204058</v>
       </c>
       <c r="AL19">
-        <v>-38.101259</v>
+        <v>-38.137175</v>
       </c>
       <c r="AM19">
         <v>0.018289</v>
@@ -21887,7 +21899,7 @@
         <v>-0.20399</v>
       </c>
       <c r="AT19">
-        <v>-11.613285</v>
+        <v>-11.624234</v>
       </c>
     </row>
     <row r="20" spans="1:46">
@@ -21922,7 +21934,7 @@
         <v>359</v>
       </c>
       <c r="K20" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="L20">
         <v>100</v>
@@ -21979,7 +21991,7 @@
         <v>-11.03366667</v>
       </c>
       <c r="AD20" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE20">
         <v>0.093333</v>
@@ -22003,7 +22015,7 @@
         <v>0.16662</v>
       </c>
       <c r="AL20">
-        <v>-37.201341</v>
+        <v>-37.290746</v>
       </c>
       <c r="AM20">
         <v>0.028456</v>
@@ -22027,7 +22039,7 @@
         <v>0.166908</v>
       </c>
       <c r="AT20">
-        <v>-11.338987</v>
+        <v>-11.366239</v>
       </c>
     </row>
     <row r="21" spans="1:46">
@@ -22062,7 +22074,7 @@
         <v>360</v>
       </c>
       <c r="K21" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="L21">
         <v>121</v>
@@ -22119,7 +22131,7 @@
         <v>-10.88133333</v>
       </c>
       <c r="AD21" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE21">
         <v>0.016667</v>
@@ -22143,7 +22155,7 @@
         <v>-0.694296</v>
       </c>
       <c r="AL21">
-        <v>-36.40851</v>
+        <v>-36.535545</v>
       </c>
       <c r="AM21">
         <v>0.005078</v>
@@ -22167,7 +22179,7 @@
         <v>-0.694285</v>
       </c>
       <c r="AT21">
-        <v>-11.097326</v>
+        <v>-11.136048</v>
       </c>
     </row>
     <row r="22" spans="1:46">
@@ -22202,7 +22214,7 @@
         <v>361</v>
       </c>
       <c r="K22" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="L22">
         <v>128</v>
@@ -22259,7 +22271,7 @@
         <v>-10.71866667</v>
       </c>
       <c r="AD22" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE22">
         <v>0.017778</v>
@@ -22283,7 +22295,7 @@
         <v>-0.656907</v>
       </c>
       <c r="AL22">
-        <v>-35.683457</v>
+        <v>-35.827562</v>
       </c>
       <c r="AM22">
         <v>0.005422</v>
@@ -22307,7 +22319,7 @@
         <v>-0.656704</v>
       </c>
       <c r="AT22">
-        <v>-10.876324</v>
+        <v>-10.920249</v>
       </c>
     </row>
     <row r="23" spans="1:46">
@@ -22342,7 +22354,7 @@
         <v>362</v>
       </c>
       <c r="K23" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="L23">
         <v>116</v>
@@ -22399,7 +22411,7 @@
         <v>-10.15</v>
       </c>
       <c r="AD23" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE23">
         <v>0.062222</v>
@@ -22423,7 +22435,7 @@
         <v>-0.123269</v>
       </c>
       <c r="AL23">
-        <v>-35.018554</v>
+        <v>-35.158521</v>
       </c>
       <c r="AM23">
         <v>0.018956</v>
@@ -22447,7 +22459,7 @@
         <v>-0.123614</v>
       </c>
       <c r="AT23">
-        <v>-10.67365</v>
+        <v>-10.716314</v>
       </c>
     </row>
     <row r="24" spans="1:46">
@@ -22482,7 +22494,7 @@
         <v>363</v>
       </c>
       <c r="K24" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="L24">
         <v>114</v>
@@ -22539,7 +22551,7 @@
         <v>-10.18033333</v>
       </c>
       <c r="AD24" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE24">
         <v>-0.003333</v>
@@ -22563,7 +22575,7 @@
         <v>-0.887807</v>
       </c>
       <c r="AL24">
-        <v>-34.349126</v>
+        <v>-34.465909</v>
       </c>
       <c r="AM24">
         <v>-0.001011</v>
@@ -22587,7 +22599,7 @@
         <v>-0.887548</v>
       </c>
       <c r="AT24">
-        <v>-10.469601</v>
+        <v>-10.505198</v>
       </c>
     </row>
     <row r="25" spans="1:46">
@@ -22622,7 +22634,7 @@
         <v>364</v>
       </c>
       <c r="K25" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="L25">
         <v>121</v>
@@ -22679,7 +22691,7 @@
         <v>-10.414</v>
       </c>
       <c r="AD25" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE25">
         <v>-0.025556</v>
@@ -22703,7 +22715,7 @@
         <v>-1.10341</v>
       </c>
       <c r="AL25">
-        <v>-33.643453</v>
+        <v>-33.720221</v>
       </c>
       <c r="AM25">
         <v>-0.007789</v>
@@ -22727,7 +22739,7 @@
         <v>-1.103299</v>
       </c>
       <c r="AT25">
-        <v>-10.254506</v>
+        <v>-10.277906</v>
       </c>
     </row>
     <row r="26" spans="1:46">
@@ -22762,7 +22774,7 @@
         <v>365</v>
       </c>
       <c r="K26" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="L26">
         <v>106</v>
@@ -22819,7 +22831,7 @@
         <v>-9.967000000000001</v>
       </c>
       <c r="AD26" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE26">
         <v>0.048889</v>
@@ -22843,7 +22855,7 @@
         <v>-0.189711</v>
       </c>
       <c r="AL26">
-        <v>-32.937423</v>
+        <v>-32.965625</v>
       </c>
       <c r="AM26">
         <v>0.0149</v>
@@ -22867,7 +22879,7 @@
         <v>-0.189737</v>
       </c>
       <c r="AT26">
-        <v>-10.039304</v>
+        <v>-10.0479</v>
       </c>
     </row>
     <row r="27" spans="1:46">
@@ -22902,7 +22914,7 @@
         <v>366</v>
       </c>
       <c r="K27" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="L27">
         <v>118</v>
@@ -22959,7 +22971,7 @@
         <v>-9.99733333</v>
       </c>
       <c r="AD27" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE27">
         <v>-0.003333</v>
@@ -22983,7 +22995,7 @@
         <v>-0.813397</v>
       </c>
       <c r="AL27">
-        <v>-32.194725</v>
+        <v>-32.17043</v>
       </c>
       <c r="AM27">
         <v>-0.001011</v>
@@ -23007,7 +23019,7 @@
         <v>-0.813111</v>
       </c>
       <c r="AT27">
-        <v>-9.81293</v>
+        <v>-9.805524</v>
       </c>
     </row>
     <row r="28" spans="1:46">
@@ -23042,7 +23054,7 @@
         <v>367</v>
       </c>
       <c r="K28" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="L28">
         <v>112</v>
@@ -23099,7 +23111,7 @@
         <v>-10.028</v>
       </c>
       <c r="AD28" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE28">
         <v>-0.003333</v>
@@ -23123,7 +23135,7 @@
         <v>-0.787869</v>
       </c>
       <c r="AL28">
-        <v>-31.41638</v>
+        <v>-31.342354</v>
       </c>
       <c r="AM28">
         <v>-0.001022</v>
@@ -23147,7 +23159,7 @@
         <v>-0.788022</v>
       </c>
       <c r="AT28">
-        <v>-9.575689000000001</v>
+        <v>-9.553124</v>
       </c>
     </row>
     <row r="29" spans="1:46">
@@ -23182,7 +23194,7 @@
         <v>368</v>
       </c>
       <c r="K29" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="L29">
         <v>98</v>
@@ -23239,7 +23251,7 @@
         <v>-9.50966667</v>
       </c>
       <c r="AD29" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE29">
         <v>0.056667</v>
@@ -23263,7 +23275,7 @@
         <v>-0.027758</v>
       </c>
       <c r="AL29">
-        <v>-30.652881</v>
+        <v>-30.540232</v>
       </c>
       <c r="AM29">
         <v>0.017278</v>
@@ -23287,7 +23299,7 @@
         <v>-0.027488</v>
       </c>
       <c r="AT29">
-        <v>-9.342978</v>
+        <v>-9.308641</v>
       </c>
     </row>
     <row r="30" spans="1:46">
@@ -23322,7 +23334,7 @@
         <v>369</v>
       </c>
       <c r="K30" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="L30">
         <v>115</v>
@@ -23379,7 +23391,7 @@
         <v>-9.276</v>
       </c>
       <c r="AD30" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE30">
         <v>0.025556</v>
@@ -23403,7 +23415,7 @@
         <v>-0.420536</v>
       </c>
       <c r="AL30">
-        <v>-29.89232</v>
+        <v>-29.754453</v>
       </c>
       <c r="AM30">
         <v>0.007789</v>
@@ -23427,7 +23439,7 @@
         <v>-0.420509</v>
       </c>
       <c r="AT30">
-        <v>-9.111164</v>
+        <v>-9.069140000000001</v>
       </c>
     </row>
     <row r="31" spans="1:46">
@@ -23462,7 +23474,7 @@
         <v>370</v>
       </c>
       <c r="K31" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="L31">
         <v>107</v>
@@ -23519,7 +23531,7 @@
         <v>-9.022</v>
       </c>
       <c r="AD31" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE31">
         <v>0.027778</v>
@@ -23543,7 +23555,7 @@
         <v>-0.383792</v>
       </c>
       <c r="AL31">
-        <v>-29.146566</v>
+        <v>-28.998794</v>
       </c>
       <c r="AM31">
         <v>0.008467000000000001</v>
@@ -23567,7 +23579,7 @@
         <v>-0.383759</v>
       </c>
       <c r="AT31">
-        <v>-8.883864000000001</v>
+        <v>-8.838820999999999</v>
       </c>
     </row>
     <row r="32" spans="1:46">
@@ -23602,7 +23614,7 @@
         <v>371</v>
       </c>
       <c r="K32" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="L32">
         <v>108</v>
@@ -23659,7 +23671,7 @@
         <v>-8.625999999999999</v>
       </c>
       <c r="AD32" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE32">
         <v>0.043333</v>
@@ -23683,7 +23695,7 @@
         <v>-0.173692</v>
       </c>
       <c r="AL32">
-        <v>-28.436669</v>
+        <v>-28.29408</v>
       </c>
       <c r="AM32">
         <v>0.0132</v>
@@ -23707,7 +23719,7 @@
         <v>-0.174042</v>
       </c>
       <c r="AT32">
-        <v>-8.667486999999999</v>
+        <v>-8.624025</v>
       </c>
     </row>
     <row r="33" spans="1:46">
@@ -23742,7 +23754,7 @@
         <v>372</v>
       </c>
       <c r="K33" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="L33">
         <v>107</v>
@@ -23799,7 +23811,7 @@
         <v>-8.199</v>
       </c>
       <c r="AD33" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE33">
         <v>0.046667</v>
@@ -23823,7 +23835,7 @@
         <v>-0.126482</v>
       </c>
       <c r="AL33">
-        <v>-27.772165</v>
+        <v>-27.647541</v>
       </c>
       <c r="AM33">
         <v>0.014233</v>
@@ -23847,7 +23859,7 @@
         <v>-0.126101</v>
       </c>
       <c r="AT33">
-        <v>-8.464953</v>
+        <v>-8.426966</v>
       </c>
     </row>
     <row r="34" spans="1:46">
@@ -23882,7 +23894,7 @@
         <v>373</v>
       </c>
       <c r="K34" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="L34">
         <v>111</v>
@@ -23939,7 +23951,7 @@
         <v>-8.128</v>
       </c>
       <c r="AD34" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE34">
         <v>0.007778</v>
@@ -23963,7 +23975,7 @@
         <v>-0.647413</v>
       </c>
       <c r="AL34">
-        <v>-27.129718</v>
+        <v>-27.034078</v>
       </c>
       <c r="AM34">
         <v>0.002367</v>
@@ -23987,7 +23999,7 @@
         <v>-0.647558</v>
       </c>
       <c r="AT34">
-        <v>-8.269138999999999</v>
+        <v>-8.239986999999999</v>
       </c>
     </row>
     <row r="35" spans="1:46">
@@ -24022,7 +24034,7 @@
         <v>374</v>
       </c>
       <c r="K35" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="L35">
         <v>104</v>
@@ -24079,7 +24091,7 @@
         <v>-8.22966667</v>
       </c>
       <c r="AD35" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE35">
         <v>-0.011111</v>
@@ -24103,7 +24115,7 @@
         <v>-0.885152</v>
       </c>
       <c r="AL35">
-        <v>-26.501306</v>
+        <v>-26.443954</v>
       </c>
       <c r="AM35">
         <v>-0.003389</v>
@@ -24127,7 +24139,7 @@
         <v>-0.885178</v>
       </c>
       <c r="AT35">
-        <v>-8.077601</v>
+        <v>-8.06012</v>
       </c>
     </row>
     <row r="36" spans="1:46">
@@ -24162,7 +24174,7 @@
         <v>375</v>
       </c>
       <c r="K36" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="L36">
         <v>114</v>
@@ -24219,7 +24231,7 @@
         <v>-7.91466667</v>
       </c>
       <c r="AD36" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE36">
         <v>0.034444</v>
@@ -24243,7 +24255,7 @@
         <v>-0.246081</v>
       </c>
       <c r="AL36">
-        <v>-25.922081</v>
+        <v>-25.907004</v>
       </c>
       <c r="AM36">
         <v>0.0105</v>
@@ -24267,7 +24279,7 @@
         <v>-0.245985</v>
       </c>
       <c r="AT36">
-        <v>-7.901055</v>
+        <v>-7.89646</v>
       </c>
     </row>
     <row r="37" spans="1:46">
@@ -24302,7 +24314,7 @@
         <v>376</v>
       </c>
       <c r="K37" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="L37">
         <v>115</v>
@@ -24359,7 +24371,7 @@
         <v>-7.559</v>
       </c>
       <c r="AD37" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE37">
         <v>0.038889</v>
@@ -24383,7 +24395,7 @@
         <v>-0.180549</v>
       </c>
       <c r="AL37">
-        <v>-25.39466</v>
+        <v>-25.421734</v>
       </c>
       <c r="AM37">
         <v>0.011856</v>
@@ -24407,7 +24419,7 @@
         <v>-0.18044</v>
       </c>
       <c r="AT37">
-        <v>-7.7403</v>
+        <v>-7.748553</v>
       </c>
     </row>
     <row r="38" spans="1:46">
@@ -24442,7 +24454,7 @@
         <v>377</v>
       </c>
       <c r="K38" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="L38">
         <v>111</v>
@@ -24499,7 +24511,7 @@
         <v>-7.53866667</v>
       </c>
       <c r="AD38" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE38">
         <v>0.002222</v>
@@ -24523,7 +24535,7 @@
         <v>-0.692309</v>
       </c>
       <c r="AL38">
-        <v>-24.895441</v>
+        <v>-24.962994</v>
       </c>
       <c r="AM38">
         <v>0.000678</v>
@@ -24547,7 +24559,7 @@
         <v>-0.692235</v>
       </c>
       <c r="AT38">
-        <v>-7.58814</v>
+        <v>-7.608731</v>
       </c>
     </row>
     <row r="39" spans="1:46">
@@ -24582,7 +24594,7 @@
         <v>378</v>
       </c>
       <c r="K39" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="L39">
         <v>108</v>
@@ -24639,7 +24651,7 @@
         <v>-7.56933333</v>
       </c>
       <c r="AD39" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE39">
         <v>-0.003333</v>
@@ -24663,7 +24675,7 @@
         <v>-0.7561600000000001</v>
       </c>
       <c r="AL39">
-        <v>-24.421956</v>
+        <v>-24.525338</v>
       </c>
       <c r="AM39">
         <v>-0.001022</v>
@@ -24687,7 +24699,7 @@
         <v>-0.75637</v>
       </c>
       <c r="AT39">
-        <v>-7.44382</v>
+        <v>-7.475333</v>
       </c>
     </row>
     <row r="40" spans="1:46">
@@ -24722,7 +24734,7 @@
         <v>379</v>
       </c>
       <c r="K40" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="L40">
         <v>109</v>
@@ -24779,7 +24791,7 @@
         <v>-7.20333333</v>
       </c>
       <c r="AD40" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE40">
         <v>0.04</v>
@@ -24803,7 +24815,7 @@
         <v>-0.124246</v>
       </c>
       <c r="AL40">
-        <v>-23.997298</v>
+        <v>-24.127539</v>
       </c>
       <c r="AM40">
         <v>0.0122</v>
@@ -24827,7 +24839,7 @@
         <v>-0.123857</v>
       </c>
       <c r="AT40">
-        <v>-7.314386</v>
+        <v>-7.354086</v>
       </c>
     </row>
     <row r="41" spans="1:46">
@@ -24862,7 +24874,7 @@
         <v>380</v>
       </c>
       <c r="K41" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="L41">
         <v>109</v>
@@ -24919,7 +24931,7 @@
         <v>-7.00033333</v>
       </c>
       <c r="AD41" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE41">
         <v>0.022222</v>
@@ -24943,7 +24955,7 @@
         <v>-0.380729</v>
       </c>
       <c r="AL41">
-        <v>-23.608505</v>
+        <v>-23.755957</v>
       </c>
       <c r="AM41">
         <v>0.006767</v>
@@ -24967,7 +24979,7 @@
         <v>-0.381011</v>
       </c>
       <c r="AT41">
-        <v>-7.19588</v>
+        <v>-7.240825</v>
       </c>
     </row>
     <row r="42" spans="1:46">
@@ -25002,7 +25014,7 @@
         <v>381</v>
       </c>
       <c r="K42" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="L42">
         <v>110</v>
@@ -25059,7 +25071,7 @@
         <v>-6.94933333</v>
       </c>
       <c r="AD42" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE42">
         <v>0.005556</v>
@@ -25083,7 +25095,7 @@
         <v>-0.618387</v>
       </c>
       <c r="AL42">
-        <v>-23.245175</v>
+        <v>-23.399546</v>
       </c>
       <c r="AM42">
         <v>0.0017</v>
@@ -25107,7 +25119,7 @@
         <v>-0.618036</v>
       </c>
       <c r="AT42">
-        <v>-7.085138</v>
+        <v>-7.132192</v>
       </c>
     </row>
     <row r="43" spans="1:46">
@@ -25142,7 +25154,7 @@
         <v>382</v>
       </c>
       <c r="K43" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="L43">
         <v>116</v>
@@ -25199,7 +25211,7 @@
         <v>-6.97</v>
       </c>
       <c r="AD43" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE43">
         <v>-0.002222</v>
@@ -25223,7 +25235,7 @@
         <v>-0.7216399999999999</v>
       </c>
       <c r="AL43">
-        <v>-22.902624</v>
+        <v>-23.05291</v>
       </c>
       <c r="AM43">
         <v>-0.0006890000000000001</v>
@@ -25247,7 +25259,7 @@
         <v>-0.722151</v>
       </c>
       <c r="AT43">
-        <v>-6.980724</v>
+        <v>-7.026533</v>
       </c>
     </row>
     <row r="44" spans="1:46">
@@ -25282,7 +25294,7 @@
         <v>383</v>
       </c>
       <c r="K44" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="L44">
         <v>121</v>
@@ -25339,7 +25351,7 @@
         <v>-6.89866667</v>
       </c>
       <c r="AD44" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE44">
         <v>0.007778</v>
@@ -25363,7 +25375,7 @@
         <v>-0.561558</v>
       </c>
       <c r="AL44">
-        <v>-22.584244</v>
+        <v>-22.719492</v>
       </c>
       <c r="AM44">
         <v>0.002378</v>
@@ -25387,7 +25399,7 @@
         <v>-0.561146</v>
       </c>
       <c r="AT44">
-        <v>-6.88368</v>
+        <v>-6.924905</v>
       </c>
     </row>
     <row r="45" spans="1:46">
@@ -25422,7 +25434,7 @@
         <v>384</v>
       </c>
       <c r="K45" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="L45">
         <v>118</v>
@@ -25479,7 +25491,7 @@
         <v>-6.82733333</v>
       </c>
       <c r="AD45" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE45">
         <v>0.007778</v>
@@ -25503,7 +25515,7 @@
         <v>-0.55307</v>
       </c>
       <c r="AL45">
-        <v>-22.288591</v>
+        <v>-22.398804</v>
       </c>
       <c r="AM45">
         <v>0.002378</v>
@@ -25527,7 +25539,7 @@
         <v>-0.5526529999999999</v>
       </c>
       <c r="AT45">
-        <v>-6.793566</v>
+        <v>-6.82716</v>
       </c>
     </row>
     <row r="46" spans="1:46">
@@ -25562,7 +25574,7 @@
         <v>385</v>
       </c>
       <c r="K46" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="L46">
         <v>116</v>
@@ -25619,7 +25631,7 @@
         <v>-6.77666667</v>
       </c>
       <c r="AD46" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE46">
         <v>0.005556</v>
@@ -25643,7 +25655,7 @@
         <v>-0.578359</v>
       </c>
       <c r="AL46">
-        <v>-22.013571</v>
+        <v>-22.090273</v>
       </c>
       <c r="AM46">
         <v>0.001689</v>
@@ -25667,7 +25679,7 @@
         <v>-0.57853</v>
       </c>
       <c r="AT46">
-        <v>-6.70974</v>
+        <v>-6.733119</v>
       </c>
     </row>
     <row r="47" spans="1:46">
@@ -25702,7 +25714,7 @@
         <v>386</v>
       </c>
       <c r="K47" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="L47">
         <v>117</v>
@@ -25759,7 +25771,7 @@
         <v>-6.736</v>
       </c>
       <c r="AD47" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE47">
         <v>0.004444</v>
@@ -25783,7 +25795,7 @@
         <v>-0.586728</v>
       </c>
       <c r="AL47">
-        <v>-21.757838</v>
+        <v>-21.794646</v>
       </c>
       <c r="AM47">
         <v>0.001356</v>
@@ -25807,7 +25819,7 @@
         <v>-0.5865939999999999</v>
       </c>
       <c r="AT47">
-        <v>-6.631792</v>
+        <v>-6.643012</v>
       </c>
     </row>
     <row r="48" spans="1:46">
@@ -25842,7 +25854,7 @@
         <v>387</v>
       </c>
       <c r="K48" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="L48">
         <v>128</v>
@@ -25899,7 +25911,7 @@
         <v>-6.777</v>
       </c>
       <c r="AD48" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE48">
         <v>-0.004444</v>
@@ -25923,7 +25935,7 @@
         <v>-0.713557</v>
       </c>
       <c r="AL48">
-        <v>-21.517856</v>
+        <v>-21.510469</v>
       </c>
       <c r="AM48">
         <v>-0.001367</v>
@@ -25947,7 +25959,7 @@
         <v>-0.714139</v>
       </c>
       <c r="AT48">
-        <v>-6.558642</v>
+        <v>-6.556389</v>
       </c>
     </row>
     <row r="49" spans="1:46">
@@ -25982,7 +25994,7 @@
         <v>388</v>
       </c>
       <c r="K49" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="L49">
         <v>130</v>
@@ -26039,7 +26051,7 @@
         <v>-6.38033333</v>
       </c>
       <c r="AD49" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE49">
         <v>0.043333</v>
@@ -26063,7 +26075,7 @@
         <v>0.035909</v>
       </c>
       <c r="AL49">
-        <v>-21.307413</v>
+        <v>-21.257403</v>
       </c>
       <c r="AM49">
         <v>0.013222</v>
@@ -26087,7 +26099,7 @@
         <v>0.036648</v>
       </c>
       <c r="AT49">
-        <v>-6.4945</v>
+        <v>-6.479256</v>
       </c>
     </row>
     <row r="50" spans="1:46">
@@ -26122,7 +26134,7 @@
         <v>389</v>
       </c>
       <c r="K50" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="L50">
         <v>126</v>
@@ -26179,7 +26191,7 @@
         <v>-6.44133333</v>
       </c>
       <c r="AD50" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE50">
         <v>-0.006667</v>
@@ -26203,7 +26215,7 @@
         <v>-0.745177</v>
       </c>
       <c r="AL50">
-        <v>-21.109869</v>
+        <v>-21.018712</v>
       </c>
       <c r="AM50">
         <v>-0.002033</v>
@@ -26227,7 +26239,7 @@
         <v>-0.745188</v>
       </c>
       <c r="AT50">
-        <v>-6.434289</v>
+        <v>-6.406503</v>
       </c>
     </row>
     <row r="51" spans="1:46">
@@ -26262,7 +26274,7 @@
         <v>390</v>
       </c>
       <c r="K51" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="L51">
         <v>121</v>
@@ -26319,7 +26331,7 @@
         <v>-6.63466667</v>
       </c>
       <c r="AD51" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE51">
         <v>-0.021111</v>
@@ -26343,7 +26355,7 @@
         <v>-0.956239</v>
       </c>
       <c r="AL51">
-        <v>-20.921589</v>
+        <v>-20.793113</v>
       </c>
       <c r="AM51">
         <v>-0.006444</v>
@@ -26367,7 +26379,7 @@
         <v>-0.956613</v>
       </c>
       <c r="AT51">
-        <v>-6.376899</v>
+        <v>-6.337738</v>
       </c>
     </row>
     <row r="52" spans="1:46">
@@ -26402,7 +26414,7 @@
         <v>391</v>
       </c>
       <c r="K52" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="L52">
         <v>113</v>
@@ -26459,7 +26471,7 @@
         <v>-6.25866667</v>
       </c>
       <c r="AD52" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE52">
         <v>0.041111</v>
@@ -26483,7 +26495,7 @@
         <v>0.03609</v>
       </c>
       <c r="AL52">
-        <v>-20.757441</v>
+        <v>-20.601214</v>
       </c>
       <c r="AM52">
         <v>0.012533</v>
@@ -26507,7 +26519,7 @@
         <v>0.036222</v>
       </c>
       <c r="AT52">
-        <v>-6.326867</v>
+        <v>-6.279246</v>
       </c>
     </row>
     <row r="53" spans="1:46">
@@ -26542,7 +26554,7 @@
         <v>392</v>
       </c>
       <c r="K53" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="L53">
         <v>122</v>
@@ -26599,7 +26611,7 @@
         <v>-6.37</v>
       </c>
       <c r="AD53" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE53">
         <v>-0.012222</v>
@@ -26623,7 +26635,7 @@
         <v>-0.810144</v>
       </c>
       <c r="AL53">
-        <v>-20.60279</v>
+        <v>-20.428176</v>
       </c>
       <c r="AM53">
         <v>-0.003711</v>
@@ -26647,7 +26659,7 @@
         <v>-0.809317</v>
       </c>
       <c r="AT53">
-        <v>-6.279731</v>
+        <v>-6.226507</v>
       </c>
     </row>
     <row r="54" spans="1:46">
@@ -26682,7 +26694,7 @@
         <v>393</v>
       </c>
       <c r="K54" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="L54">
         <v>128</v>
@@ -26739,7 +26751,7 @@
         <v>-6.269</v>
       </c>
       <c r="AD54" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE54">
         <v>0.011111</v>
@@ -26763,7 +26775,7 @@
         <v>-0.427903</v>
       </c>
       <c r="AL54">
-        <v>-20.461428</v>
+        <v>-20.280308</v>
       </c>
       <c r="AM54">
         <v>0.003367</v>
@@ -26787,7 +26799,7 @@
         <v>-0.428915</v>
       </c>
       <c r="AT54">
-        <v>-6.236643</v>
+        <v>-6.181435</v>
       </c>
     </row>
     <row r="55" spans="1:46">
@@ -26822,7 +26834,7 @@
         <v>394</v>
       </c>
       <c r="K55" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="L55">
         <v>129</v>
@@ -26879,7 +26891,7 @@
         <v>-6.08566667</v>
       </c>
       <c r="AD55" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE55">
         <v>0.02</v>
@@ -26903,7 +26915,7 @@
         <v>-0.280121</v>
       </c>
       <c r="AL55">
-        <v>-20.332604</v>
+        <v>-20.157327</v>
       </c>
       <c r="AM55">
         <v>0.006111</v>
@@ -26927,7 +26939,7 @@
         <v>-0.279277</v>
       </c>
       <c r="AT55">
-        <v>-6.197378</v>
+        <v>-6.143952</v>
       </c>
     </row>
     <row r="56" spans="1:46">
@@ -26962,7 +26974,7 @@
         <v>395</v>
       </c>
       <c r="K56" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="L56">
         <v>134</v>
@@ -27019,7 +27031,7 @@
         <v>-6.12666667</v>
       </c>
       <c r="AD56" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE56">
         <v>-0.004444</v>
@@ -27043,7 +27055,7 @@
         <v>-0.67306</v>
       </c>
       <c r="AL56">
-        <v>-20.208862</v>
+        <v>-20.051985</v>
       </c>
       <c r="AM56">
         <v>-0.001367</v>
@@ -27067,7 +27079,7 @@
         <v>-0.673664</v>
       </c>
       <c r="AT56">
-        <v>-6.159661</v>
+        <v>-6.111844</v>
       </c>
     </row>
     <row r="57" spans="1:46">
@@ -27102,7 +27114,7 @@
         <v>396</v>
       </c>
       <c r="K57" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="L57">
         <v>131</v>
@@ -27159,7 +27171,7 @@
         <v>-5.87233333</v>
       </c>
       <c r="AD57" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE57">
         <v>0.027778</v>
@@ -27183,7 +27195,7 @@
         <v>-0.138976</v>
       </c>
       <c r="AL57">
-        <v>-20.093014</v>
+        <v>-19.965188</v>
       </c>
       <c r="AM57">
         <v>0.008477999999999999</v>
@@ -27207,7 +27219,7 @@
         <v>-0.138337</v>
       </c>
       <c r="AT57">
-        <v>-6.124351</v>
+        <v>-6.085389</v>
       </c>
     </row>
     <row r="58" spans="1:46">
@@ -27242,7 +27254,7 @@
         <v>397</v>
       </c>
       <c r="K58" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="L58">
         <v>126</v>
@@ -27299,7 +27311,7 @@
         <v>-6.00466667</v>
       </c>
       <c r="AD58" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE58">
         <v>-0.014444</v>
@@ -27323,7 +27335,7 @@
         <v>-0.830773</v>
       </c>
       <c r="AL58">
-        <v>-19.973887</v>
+        <v>-19.886114</v>
       </c>
       <c r="AM58">
         <v>-0.004411</v>
@@ -27347,7 +27359,7 @@
         <v>-0.831147</v>
       </c>
       <c r="AT58">
-        <v>-6.088041</v>
+        <v>-6.061288</v>
       </c>
     </row>
     <row r="59" spans="1:46">
@@ -27382,7 +27394,7 @@
         <v>398</v>
       </c>
       <c r="K59" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="L59">
         <v>126</v>
@@ -27439,7 +27451,7 @@
         <v>-6.08566667</v>
       </c>
       <c r="AD59" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE59">
         <v>-0.008888999999999999</v>
@@ -27463,7 +27475,7 @@
         <v>-0.727916</v>
       </c>
       <c r="AL59">
-        <v>-19.84828</v>
+        <v>-19.809671</v>
       </c>
       <c r="AM59">
         <v>-0.0027</v>
@@ -27487,7 +27499,7 @@
         <v>-0.727303</v>
       </c>
       <c r="AT59">
-        <v>-6.049757</v>
+        <v>-6.037989</v>
       </c>
     </row>
     <row r="60" spans="1:46">
@@ -27522,7 +27534,7 @@
         <v>399</v>
       </c>
       <c r="K60" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="L60">
         <v>130</v>
@@ -27579,7 +27591,7 @@
         <v>-6.06566667</v>
       </c>
       <c r="AD60" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE60">
         <v>0.002222</v>
@@ -27603,7 +27615,7 @@
         <v>-0.535231</v>
       </c>
       <c r="AL60">
-        <v>-19.713477</v>
+        <v>-19.729464</v>
       </c>
       <c r="AM60">
         <v>0.0006669999999999999</v>
@@ -27627,7 +27639,7 @@
         <v>-0.535752</v>
       </c>
       <c r="AT60">
-        <v>-6.008667</v>
+        <v>-6.013542</v>
       </c>
     </row>
     <row r="61" spans="1:46">
@@ -27662,7 +27674,7 @@
         <v>400</v>
       </c>
       <c r="K61" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="L61">
         <v>125</v>
@@ -27719,7 +27731,7 @@
         <v>-6.06533333</v>
       </c>
       <c r="AD61" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE61">
         <v>0</v>
@@ -27743,7 +27755,7 @@
         <v>-0.566404</v>
       </c>
       <c r="AL61">
-        <v>-19.563965</v>
+        <v>-19.636383</v>
       </c>
       <c r="AM61">
         <v>1.1E-05</v>
@@ -27767,7 +27779,7 @@
         <v>-0.565761</v>
       </c>
       <c r="AT61">
-        <v>-5.963097</v>
+        <v>-5.985172</v>
       </c>
     </row>
     <row r="62" spans="1:46">
@@ -27802,7 +27814,7 @@
         <v>401</v>
       </c>
       <c r="K62" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="L62">
         <v>124</v>
@@ -27859,7 +27871,7 @@
         <v>-6.025</v>
       </c>
       <c r="AD62" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE62">
         <v>0.004444</v>
@@ -27883,7 +27895,7 @@
         <v>-0.485782</v>
       </c>
       <c r="AL62">
-        <v>-19.395735</v>
+        <v>-19.521734</v>
       </c>
       <c r="AM62">
         <v>0.001344</v>
@@ -27907,7 +27919,7 @@
         <v>-0.486324</v>
       </c>
       <c r="AT62">
-        <v>-5.911818</v>
+        <v>-5.950226</v>
       </c>
     </row>
     <row r="63" spans="1:46">
@@ -27942,7 +27954,7 @@
         <v>402</v>
       </c>
       <c r="K63" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="L63">
         <v>122</v>
@@ -27999,7 +28011,7 @@
         <v>-5.93333333</v>
       </c>
       <c r="AD63" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE63">
         <v>0.01</v>
@@ -28023,7 +28035,7 @@
         <v>-0.387009</v>
       </c>
       <c r="AL63">
-        <v>-19.206052</v>
+        <v>-19.377932</v>
       </c>
       <c r="AM63">
         <v>0.003056</v>
@@ -28047,7 +28059,7 @@
         <v>-0.386504</v>
       </c>
       <c r="AT63">
-        <v>-5.854003</v>
+        <v>-5.906395</v>
       </c>
     </row>
     <row r="64" spans="1:46">
@@ -28082,7 +28094,7 @@
         <v>403</v>
       </c>
       <c r="K64" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="L64">
         <v>136</v>
@@ -28139,7 +28151,7 @@
         <v>-6.13666667</v>
       </c>
       <c r="AD64" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE64">
         <v>-0.022222</v>
@@ -28163,7 +28175,7 @@
         <v>-0.928369</v>
       </c>
       <c r="AL64">
-        <v>-18.980391</v>
+        <v>-19.187816</v>
       </c>
       <c r="AM64">
         <v>-0.006778</v>
@@ -28187,7 +28199,7 @@
         <v>-0.928596</v>
       </c>
       <c r="AT64">
-        <v>-5.78522</v>
+        <v>-5.848447</v>
       </c>
     </row>
     <row r="65" spans="1:46">
@@ -28222,7 +28234,7 @@
         <v>404</v>
       </c>
       <c r="K65" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="L65">
         <v>128</v>
@@ -28279,7 +28291,7 @@
         <v>-6.16733333</v>
       </c>
       <c r="AD65" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE65">
         <v>-0.003333</v>
@@ -28303,7 +28315,7 @@
         <v>-0.595871</v>
       </c>
       <c r="AL65">
-        <v>-18.719966</v>
+        <v>-18.946423</v>
       </c>
       <c r="AM65">
         <v>-0.001022</v>
@@ -28327,7 +28339,7 @@
         <v>-0.596164</v>
       </c>
       <c r="AT65">
-        <v>-5.705839</v>
+        <v>-5.774866</v>
       </c>
     </row>
     <row r="66" spans="1:46">
@@ -28362,7 +28374,7 @@
         <v>405</v>
       </c>
       <c r="K66" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="L66">
         <v>136</v>
@@ -28419,7 +28431,7 @@
         <v>-6.20766667</v>
       </c>
       <c r="AD66" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE66">
         <v>-0.004444</v>
@@ -28443,7 +28455,7 @@
         <v>-0.608576</v>
       </c>
       <c r="AL66">
-        <v>-18.421973</v>
+        <v>-18.646977</v>
       </c>
       <c r="AM66">
         <v>-0.001344</v>
@@ -28467,7 +28479,7 @@
         <v>-0.607917</v>
       </c>
       <c r="AT66">
-        <v>-5.615011</v>
+        <v>-5.683595</v>
       </c>
     </row>
     <row r="67" spans="1:46">
@@ -28502,7 +28514,7 @@
         <v>406</v>
       </c>
       <c r="K67" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="L67">
         <v>130</v>
@@ -28559,7 +28571,7 @@
         <v>-1.31146914</v>
       </c>
       <c r="AD67" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE67">
         <v>0.003966</v>
@@ -28583,7 +28595,7 @@
         <v>-0.457643</v>
       </c>
       <c r="AL67">
-        <v>-18.148302</v>
+        <v>-18.354766</v>
       </c>
       <c r="AM67">
         <v>0.001209</v>
@@ -28607,7 +28619,7 @@
         <v>-0.457607</v>
       </c>
       <c r="AT67">
-        <v>-5.531595</v>
+        <v>-5.594527</v>
       </c>
     </row>
     <row r="68" spans="1:46">
@@ -28642,7 +28654,7 @@
         <v>407</v>
       </c>
       <c r="K68" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="L68">
         <v>132</v>
@@ -28699,7 +28711,7 @@
         <v>-6.035</v>
       </c>
       <c r="AD68" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE68">
         <v>-0.516576</v>
@@ -28723,7 +28735,7 @@
         <v>-6.1249</v>
       </c>
       <c r="AL68">
-        <v>-18.098342</v>
+        <v>-18.299934</v>
       </c>
       <c r="AM68">
         <v>-0.157451</v>
@@ -28747,7 +28759,7 @@
         <v>-6.124631</v>
       </c>
       <c r="AT68">
-        <v>-5.516368</v>
+        <v>-5.577815</v>
       </c>
     </row>
     <row r="69" spans="1:46">
@@ -28782,7 +28794,7 @@
         <v>408</v>
       </c>
       <c r="K69" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="L69">
         <v>139</v>
@@ -28839,7 +28851,7 @@
         <v>-5.76066667</v>
       </c>
       <c r="AD69" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE69">
         <v>0.03</v>
@@ -28863,7 +28875,7 @@
         <v>0.092983</v>
       </c>
       <c r="AL69">
-        <v>-17.761231</v>
+        <v>-17.919981</v>
       </c>
       <c r="AM69">
         <v>0.009143999999999999</v>
@@ -28887,7 +28899,7 @@
         <v>0.092971</v>
       </c>
       <c r="AT69">
-        <v>-5.413618</v>
+        <v>-5.462006</v>
       </c>
     </row>
     <row r="70" spans="1:46">
@@ -28922,7 +28934,7 @@
         <v>409</v>
       </c>
       <c r="K70" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="L70">
         <v>134</v>
@@ -28979,7 +28991,7 @@
         <v>-5.73533333</v>
       </c>
       <c r="AD70" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE70">
         <v>0.001389</v>
@@ -29003,7 +29015,7 @@
         <v>-0.233196</v>
       </c>
       <c r="AL70">
-        <v>-17.462291</v>
+        <v>-17.571067</v>
       </c>
       <c r="AM70">
         <v>0.000422</v>
@@ -29027,7 +29039,7 @@
         <v>-0.233249</v>
       </c>
       <c r="AT70">
-        <v>-5.322498</v>
+        <v>-5.355652</v>
       </c>
     </row>
     <row r="71" spans="1:46">
@@ -29062,7 +29074,7 @@
         <v>410</v>
       </c>
       <c r="K71" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="L71">
         <v>133</v>
@@ -29119,7 +29131,7 @@
         <v>-5.54733333</v>
       </c>
       <c r="AD71" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE71">
         <v>0.020556</v>
@@ -29143,7 +29155,7 @@
         <v>-0.011829</v>
       </c>
       <c r="AL71">
-        <v>-17.415822</v>
+        <v>-17.51601</v>
       </c>
       <c r="AM71">
         <v>0.006267</v>
@@ -29167,7 +29179,7 @@
         <v>-0.011753</v>
       </c>
       <c r="AT71">
-        <v>-5.308338</v>
+        <v>-5.338875</v>
       </c>
     </row>
     <row r="72" spans="1:46">
@@ -29202,7 +29214,7 @@
         <v>411</v>
       </c>
       <c r="K72" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="L72">
         <v>122</v>
@@ -29259,7 +29271,7 @@
         <v>-5.466</v>
       </c>
       <c r="AD72" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE72">
         <v>0.008888999999999999</v>
@@ -29283,7 +29295,7 @@
         <v>-0.146457</v>
       </c>
       <c r="AL72">
-        <v>-17.062923</v>
+        <v>-17.092235</v>
       </c>
       <c r="AM72">
         <v>0.002711</v>
@@ -29307,7 +29319,7 @@
         <v>-0.146393</v>
       </c>
       <c r="AT72">
-        <v>-5.200776</v>
+        <v>-5.20971</v>
       </c>
     </row>
     <row r="73" spans="1:46">
@@ -29342,7 +29354,7 @@
         <v>412</v>
       </c>
       <c r="K73" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="L73">
         <v>130</v>
@@ -29399,7 +29411,7 @@
         <v>-5.41516667</v>
       </c>
       <c r="AD73" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE73">
         <v>0.002778</v>
@@ -29423,7 +29435,7 @@
         <v>-0.216457</v>
       </c>
       <c r="AL73">
-        <v>-16.761197</v>
+        <v>-16.724122</v>
       </c>
       <c r="AM73">
         <v>0.000847</v>
@@ -29447,7 +29459,7 @@
         <v>-0.216431</v>
       </c>
       <c r="AT73">
-        <v>-5.108811</v>
+        <v>-5.097508</v>
       </c>
     </row>
     <row r="74" spans="1:46">
@@ -29482,7 +29494,7 @@
         <v>413</v>
       </c>
       <c r="K74" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="L74">
         <v>132</v>
@@ -29539,7 +29551,7 @@
         <v>-5.36466667</v>
       </c>
       <c r="AD74" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE74">
         <v>0.005556</v>
@@ -29563,7 +29575,7 @@
         <v>-0.182387</v>
       </c>
       <c r="AL74">
-        <v>-16.713828</v>
+        <v>-16.666034</v>
       </c>
       <c r="AM74">
         <v>0.001683</v>
@@ -29587,7 +29599,7 @@
         <v>-0.182778</v>
       </c>
       <c r="AT74">
-        <v>-5.09437</v>
+        <v>-5.079799</v>
       </c>
     </row>
     <row r="75" spans="1:46">
@@ -29622,7 +29634,7 @@
         <v>414</v>
       </c>
       <c r="K75" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="L75">
         <v>130</v>
@@ -29679,7 +29691,7 @@
         <v>-5.50666667</v>
       </c>
       <c r="AD75" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE75">
         <v>-0.015556</v>
@@ -29703,7 +29715,7 @@
         <v>-0.429624</v>
       </c>
       <c r="AL75">
-        <v>-16.364535</v>
+        <v>-16.237102</v>
       </c>
       <c r="AM75">
         <v>-0.004733</v>
@@ -29727,7 +29739,7 @@
         <v>-0.429288</v>
       </c>
       <c r="AT75">
-        <v>-4.987908</v>
+        <v>-4.949062</v>
       </c>
     </row>
     <row r="76" spans="1:46">
@@ -29762,7 +29774,7 @@
         <v>415</v>
       </c>
       <c r="K76" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="L76">
         <v>142</v>
@@ -29819,7 +29831,7 @@
         <v>-5.43566667</v>
       </c>
       <c r="AD76" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE76">
         <v>0.003889</v>
@@ -29843,7 +29855,7 @@
         <v>-0.195999</v>
       </c>
       <c r="AL76">
-        <v>-16.087974</v>
+        <v>-15.899884</v>
       </c>
       <c r="AM76">
         <v>0.001183</v>
@@ -29867,7 +29879,7 @@
         <v>-0.196087</v>
       </c>
       <c r="AT76">
-        <v>-4.903613</v>
+        <v>-4.846279</v>
       </c>
     </row>
     <row r="77" spans="1:46">
@@ -29902,7 +29914,7 @@
         <v>416</v>
       </c>
       <c r="K77" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="L77">
         <v>140</v>
@@ -29959,7 +29971,7 @@
         <v>-5.31366667</v>
       </c>
       <c r="AD77" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE77">
         <v>0.013333</v>
@@ -29983,7 +29995,7 @@
         <v>-0.081904</v>
       </c>
       <c r="AL77">
-        <v>-16.04926</v>
+        <v>-15.853152</v>
       </c>
       <c r="AM77">
         <v>0.004067</v>
@@ -30007,7 +30019,7 @@
         <v>-0.081771</v>
       </c>
       <c r="AT77">
-        <v>-4.891814</v>
+        <v>-4.832036</v>
       </c>
     </row>
     <row r="78" spans="1:46">
@@ -30042,7 +30054,7 @@
         <v>417</v>
       </c>
       <c r="K78" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="L78">
         <v>141</v>
@@ -30099,7 +30111,7 @@
         <v>-4.97833333</v>
       </c>
       <c r="AD78" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE78">
         <v>0.036667</v>
@@ -30123,7 +30135,7 @@
         <v>0.199198</v>
       </c>
       <c r="AL78">
-        <v>-15.785529</v>
+        <v>-15.540998</v>
       </c>
       <c r="AM78">
         <v>0.011178</v>
@@ -30147,7 +30159,7 @@
         <v>0.199257</v>
       </c>
       <c r="AT78">
-        <v>-4.811432</v>
+        <v>-4.736895</v>
       </c>
     </row>
     <row r="79" spans="1:46">
@@ -30182,7 +30194,7 @@
         <v>418</v>
       </c>
       <c r="K79" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="L79">
         <v>144</v>
@@ -30239,7 +30251,7 @@
         <v>-4.8565</v>
       </c>
       <c r="AD79" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE79">
         <v>0.006667</v>
@@ -30263,7 +30275,7 @@
         <v>-0.165195</v>
       </c>
       <c r="AL79">
-        <v>-15.601313</v>
+        <v>-15.334681</v>
       </c>
       <c r="AM79">
         <v>0.002031</v>
@@ -30287,7 +30299,7 @@
         <v>-0.165259</v>
       </c>
       <c r="AT79">
-        <v>-4.755282</v>
+        <v>-4.674009</v>
       </c>
     </row>
     <row r="80" spans="1:46">
@@ -30322,7 +30334,7 @@
         <v>419</v>
       </c>
       <c r="K80" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="L80">
         <v>144</v>
@@ -30379,7 +30391,7 @@
         <v>-4.71433333</v>
       </c>
       <c r="AD80" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE80">
         <v>0.015556</v>
@@ -30403,7 +30415,7 @@
         <v>-0.055849</v>
       </c>
       <c r="AL80">
-        <v>-15.574326</v>
+        <v>-15.305907</v>
       </c>
       <c r="AM80">
         <v>0.004739</v>
@@ -30427,7 +30439,7 @@
         <v>-0.05596</v>
       </c>
       <c r="AT80">
-        <v>-4.747058</v>
+        <v>-4.66524</v>
       </c>
     </row>
     <row r="81" spans="1:46">
@@ -30462,7 +30474,7 @@
         <v>420</v>
       </c>
       <c r="K81" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="L81">
         <v>146</v>
@@ -30519,7 +30531,7 @@
         <v>-4.55166667</v>
       </c>
       <c r="AD81" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE81">
         <v>0.017778</v>
@@ -30543,7 +30555,7 @@
         <v>-0.028236</v>
       </c>
       <c r="AL81">
-        <v>-15.41403</v>
+        <v>-15.149431</v>
       </c>
       <c r="AM81">
         <v>0.005422</v>
@@ -30567,7 +30579,7 @@
         <v>-0.02812</v>
       </c>
       <c r="AT81">
-        <v>-4.698201</v>
+        <v>-4.617549</v>
       </c>
     </row>
     <row r="82" spans="1:46">
@@ -30602,7 +30614,7 @@
         <v>421</v>
       </c>
       <c r="K82" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="L82">
         <v>142</v>
@@ -30659,7 +30671,7 @@
         <v>-4.37383333</v>
       </c>
       <c r="AD82" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE82">
         <v>0.009722</v>
@@ -30683,7 +30695,7 @@
         <v>-0.127502</v>
       </c>
       <c r="AL82">
-        <v>-15.322816</v>
+        <v>-15.08292</v>
       </c>
       <c r="AM82">
         <v>0.002964</v>
@@ -30707,7 +30719,7 @@
         <v>-0.127461</v>
       </c>
       <c r="AT82">
-        <v>-4.670401</v>
+        <v>-4.597279</v>
       </c>
     </row>
     <row r="83" spans="1:46">
@@ -30742,7 +30754,7 @@
         <v>422</v>
       </c>
       <c r="K83" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="L83">
         <v>150</v>
@@ -30799,7 +30811,7 @@
         <v>-4.10466667</v>
       </c>
       <c r="AD83" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE83">
         <v>0.029444</v>
@@ -30823,7 +30835,7 @@
         <v>0.118283</v>
       </c>
       <c r="AL83">
-        <v>-15.310987</v>
+        <v>-15.076997</v>
       </c>
       <c r="AM83">
         <v>0.008972000000000001</v>
@@ -30847,7 +30859,7 @@
         <v>0.118181</v>
       </c>
       <c r="AT83">
-        <v>-4.666796</v>
+        <v>-4.595474</v>
       </c>
     </row>
     <row r="84" spans="1:46">
@@ -30882,7 +30894,7 @@
         <v>423</v>
       </c>
       <c r="K84" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="L84">
         <v>141</v>
@@ -30939,7 +30951,7 @@
         <v>-4.27733333</v>
       </c>
       <c r="AD84" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE84">
         <v>-0.018889</v>
@@ -30963,7 +30975,7 @@
         <v>-0.485966</v>
       </c>
       <c r="AL84">
-        <v>-15.253446</v>
+        <v>-15.071663</v>
       </c>
       <c r="AM84">
         <v>-0.005756</v>
@@ -30987,7 +30999,7 @@
         <v>-0.485924</v>
       </c>
       <c r="AT84">
-        <v>-4.649259</v>
+        <v>-4.593851</v>
       </c>
     </row>
     <row r="85" spans="1:46">
@@ -31022,7 +31034,7 @@
         <v>424</v>
       </c>
       <c r="K85" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="L85">
         <v>149</v>
@@ -31079,7 +31091,7 @@
         <v>-4.22666667</v>
       </c>
       <c r="AD85" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE85">
         <v>0.005556</v>
@@ -31103,7 +31115,7 @@
         <v>-0.175947</v>
       </c>
       <c r="AL85">
-        <v>-15.248079</v>
+        <v>-15.075511</v>
       </c>
       <c r="AM85">
         <v>0.001689</v>
@@ -31127,7 +31139,7 @@
         <v>-0.176134</v>
       </c>
       <c r="AT85">
-        <v>-4.647623</v>
+        <v>-4.595025</v>
       </c>
     </row>
     <row r="86" spans="1:46">
@@ -31162,7 +31174,7 @@
         <v>425</v>
       </c>
       <c r="K86" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="L86">
         <v>152</v>
@@ -31219,7 +31231,7 @@
         <v>-4.247</v>
       </c>
       <c r="AD86" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE86">
         <v>-0.002222</v>
@@ -31243,7 +31255,7 @@
         <v>-0.273089</v>
       </c>
       <c r="AL86">
-        <v>-15.227833</v>
+        <v>-15.135411</v>
       </c>
       <c r="AM86">
         <v>-0.000678</v>
@@ -31267,7 +31279,7 @@
         <v>-0.273131</v>
       </c>
       <c r="AT86">
-        <v>-4.641453</v>
+        <v>-4.613286</v>
       </c>
     </row>
     <row r="87" spans="1:46">
@@ -31302,7 +31314,7 @@
         <v>426</v>
       </c>
       <c r="K87" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="L87">
         <v>148</v>
@@ -31359,7 +31371,7 @@
         <v>-4.33833333</v>
       </c>
       <c r="AD87" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE87">
         <v>-0.01</v>
@@ -31383,7 +31395,7 @@
         <v>-0.370048</v>
       </c>
       <c r="AL87">
-        <v>-15.227418</v>
+        <v>-15.150357</v>
       </c>
       <c r="AM87">
         <v>-0.003044</v>
@@ -31407,7 +31419,7 @@
         <v>-0.369872</v>
       </c>
       <c r="AT87">
-        <v>-4.641327</v>
+        <v>-4.617843</v>
       </c>
     </row>
     <row r="88" spans="1:46">
@@ -31442,7 +31454,7 @@
         <v>427</v>
       </c>
       <c r="K88" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="L88">
         <v>182</v>
@@ -31499,7 +31511,7 @@
         <v>-4.6735</v>
       </c>
       <c r="AD88" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE88">
         <v>-0.018333</v>
@@ -31523,7 +31535,7 @@
         <v>-0.473742</v>
       </c>
       <c r="AL88">
-        <v>-15.283722</v>
+        <v>-15.484274</v>
       </c>
       <c r="AM88">
         <v>-0.005586</v>
@@ -31547,7 +31559,7 @@
         <v>-0.473678</v>
       </c>
       <c r="AT88">
-        <v>-4.65849</v>
+        <v>-4.719625</v>
       </c>
     </row>
     <row r="89" spans="1:46">
@@ -31582,7 +31594,7 @@
         <v>428</v>
       </c>
       <c r="K89" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="L89">
         <v>180</v>
@@ -31639,7 +31651,7 @@
         <v>-4.75483333</v>
       </c>
       <c r="AD89" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE89">
         <v>-0.004444</v>
@@ -31663,7 +31675,7 @@
         <v>-0.292619</v>
       </c>
       <c r="AL89">
-        <v>-15.291308</v>
+        <v>-15.52001</v>
       </c>
       <c r="AM89">
         <v>-0.001356</v>
@@ -31687,7 +31699,7 @@
         <v>-0.292697</v>
       </c>
       <c r="AT89">
-        <v>-4.660803</v>
+        <v>-4.73052</v>
       </c>
     </row>
     <row r="90" spans="1:46">
@@ -31722,7 +31734,7 @@
         <v>429</v>
       </c>
       <c r="K90" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="L90">
         <v>170</v>
@@ -31779,7 +31791,7 @@
         <v>-5.19166667</v>
       </c>
       <c r="AD90" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE90">
         <v>-0.047778</v>
@@ -31803,7 +31815,7 @@
         <v>-0.846684</v>
       </c>
       <c r="AL90">
-        <v>-15.325636</v>
+        <v>-15.743305</v>
       </c>
       <c r="AM90">
         <v>-0.014561</v>
@@ -31827,7 +31839,7 @@
         <v>-0.846554</v>
       </c>
       <c r="AT90">
-        <v>-4.671267</v>
+        <v>-4.798582</v>
       </c>
     </row>
     <row r="91" spans="1:46">
@@ -31862,7 +31874,7 @@
         <v>430</v>
       </c>
       <c r="K91" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="L91">
         <v>177</v>
@@ -31919,7 +31931,7 @@
         <v>-5.09016667</v>
       </c>
       <c r="AD91" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE91">
         <v>0.005556</v>
@@ -31943,7 +31955,7 @@
         <v>-0.152488</v>
       </c>
       <c r="AL91">
-        <v>-15.294673</v>
+        <v>-15.84321</v>
       </c>
       <c r="AM91">
         <v>0.001692</v>
@@ -31967,7 +31979,7 @@
         <v>-0.15255</v>
       </c>
       <c r="AT91">
-        <v>-4.661831</v>
+        <v>-4.829034</v>
       </c>
     </row>
     <row r="92" spans="1:46">
@@ -32002,7 +32014,7 @@
         <v>431</v>
       </c>
       <c r="K92" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="L92">
         <v>166</v>
@@ -32059,7 +32071,7 @@
         <v>-4.97833333</v>
       </c>
       <c r="AD92" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE92">
         <v>0.012222</v>
@@ -32083,7 +32095,7 @@
         <v>-0.064994</v>
       </c>
       <c r="AL92">
-        <v>-15.27899</v>
+        <v>-15.846313</v>
       </c>
       <c r="AM92">
         <v>0.003728</v>
@@ -32107,7 +32119,7 @@
         <v>-0.06486699999999999</v>
       </c>
       <c r="AT92">
-        <v>-4.657051</v>
+        <v>-4.82998</v>
       </c>
     </row>
     <row r="93" spans="1:46">
@@ -32142,7 +32154,7 @@
         <v>432</v>
       </c>
       <c r="K93" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="L93">
         <v>180</v>
@@ -32199,7 +32211,7 @@
         <v>-5.36466667</v>
       </c>
       <c r="AD93" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE93">
         <v>-0.042222</v>
@@ -32223,7 +32235,7 @@
         <v>-0.773837</v>
       </c>
       <c r="AL93">
-        <v>-15.028853</v>
+        <v>-15.653805</v>
       </c>
       <c r="AM93">
         <v>-0.012878</v>
@@ -32247,7 +32259,7 @@
         <v>-0.774195</v>
       </c>
       <c r="AT93">
-        <v>-4.58081</v>
+        <v>-4.7713</v>
       </c>
     </row>
     <row r="94" spans="1:46">
@@ -32282,7 +32294,7 @@
         <v>433</v>
       </c>
       <c r="K94" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="L94">
         <v>178</v>
@@ -32339,7 +32351,7 @@
         <v>-4.70416667</v>
       </c>
       <c r="AD94" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE94">
         <v>0.036111</v>
@@ -32363,7 +32375,7 @@
         <v>0.256721</v>
       </c>
       <c r="AL94">
-        <v>-14.703288</v>
+        <v>-15.266316</v>
       </c>
       <c r="AM94">
         <v>0.011008</v>
@@ -32387,7 +32399,7 @@
         <v>0.256778</v>
       </c>
       <c r="AT94">
-        <v>-4.481581</v>
+        <v>-4.653189</v>
       </c>
     </row>
     <row r="95" spans="1:46">
@@ -32422,7 +32434,7 @@
         <v>434</v>
       </c>
       <c r="K95" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="L95">
         <v>156</v>
@@ -32479,7 +32491,7 @@
         <v>-3.69833333</v>
       </c>
       <c r="AD95" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE95">
         <v>0.11</v>
@@ -32503,7 +32515,7 @@
         <v>1.218598</v>
       </c>
       <c r="AL95">
-        <v>-14.649413</v>
+        <v>-15.197279</v>
       </c>
       <c r="AM95">
         <v>0.033528</v>
@@ -32527,7 +32539,7 @@
         <v>1.218544</v>
       </c>
       <c r="AT95">
-        <v>-4.465156</v>
+        <v>-4.63214</v>
       </c>
     </row>
     <row r="96" spans="1:46">
@@ -32562,7 +32574,7 @@
         <v>435</v>
       </c>
       <c r="K96" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="L96">
         <v>142</v>
@@ -32619,7 +32631,7 @@
         <v>-3.26133333</v>
       </c>
       <c r="AD96" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE96">
         <v>0.047778</v>
@@ -32643,7 +32655,7 @@
         <v>0.39442</v>
       </c>
       <c r="AL96">
-        <v>-14.189325</v>
+        <v>-14.578997</v>
       </c>
       <c r="AM96">
         <v>0.014567</v>
@@ -32667,7 +32679,7 @@
         <v>0.394603</v>
       </c>
       <c r="AT96">
-        <v>-4.32493</v>
+        <v>-4.443689</v>
       </c>
     </row>
     <row r="97" spans="1:46">
@@ -32702,7 +32714,7 @@
         <v>436</v>
       </c>
       <c r="K97" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="L97">
         <v>146</v>
@@ -32759,7 +32771,7 @@
         <v>-4.379</v>
       </c>
       <c r="AD97" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE97">
         <v>-0.122222</v>
@@ -32783,7 +32795,7 @@
         <v>-1.818079</v>
       </c>
       <c r="AL97">
-        <v>-13.089189</v>
+        <v>-12.998668</v>
       </c>
       <c r="AM97">
         <v>-0.037256</v>
@@ -32807,7 +32819,7 @@
         <v>-1.818092</v>
       </c>
       <c r="AT97">
-        <v>-3.989614</v>
+        <v>-3.961987</v>
       </c>
     </row>
     <row r="98" spans="1:46">
@@ -32842,7 +32854,7 @@
         <v>437</v>
       </c>
       <c r="K98" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="L98">
         <v>156</v>
@@ -32899,7 +32911,7 @@
         <v>-4.003</v>
       </c>
       <c r="AD98" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="AE98">
         <v>0.020556</v>
@@ -32923,7 +32935,7 @@
         <v>0.05191</v>
       </c>
       <c r="AL98">
-        <v>-12.830892</v>
+        <v>-12.616729</v>
       </c>
       <c r="AM98">
         <v>0.006267</v>
@@ -32947,7 +32959,287 @@
         <v>0.051972</v>
       </c>
       <c r="AT98">
-        <v>-3.910885</v>
+        <v>-3.845567</v>
+      </c>
+    </row>
+    <row r="99" spans="1:46">
+      <c r="A99" t="s">
+        <v>37</v>
+      </c>
+      <c r="B99" t="s">
+        <v>92</v>
+      </c>
+      <c r="C99" s="2">
+        <v>45969.38877582176</v>
+      </c>
+      <c r="D99" s="2">
+        <v>45969.38871527778</v>
+      </c>
+      <c r="E99">
+        <v>4606</v>
+      </c>
+      <c r="F99">
+        <v>1403.91</v>
+      </c>
+      <c r="G99">
+        <v>-968</v>
+      </c>
+      <c r="H99">
+        <v>2580</v>
+      </c>
+      <c r="I99" t="s">
+        <v>340</v>
+      </c>
+      <c r="J99" t="s">
+        <v>438</v>
+      </c>
+      <c r="K99" t="s">
+        <v>537</v>
+      </c>
+      <c r="L99">
+        <v>140</v>
+      </c>
+      <c r="M99">
+        <v>8</v>
+      </c>
+      <c r="N99">
+        <v>12.9</v>
+      </c>
+      <c r="O99">
+        <v>39.414</v>
+      </c>
+      <c r="P99">
+        <v>-102.4771666667</v>
+      </c>
+      <c r="Q99">
+        <v>101.61</v>
+      </c>
+      <c r="R99">
+        <v>163.53</v>
+      </c>
+      <c r="S99">
+        <v>40.28</v>
+      </c>
+      <c r="T99">
+        <v>4.6</v>
+      </c>
+      <c r="U99">
+        <v>277.75</v>
+      </c>
+      <c r="V99">
+        <v>86220</v>
+      </c>
+      <c r="W99">
+        <v>0.85</v>
+      </c>
+      <c r="X99">
+        <v>0.00209831</v>
+      </c>
+      <c r="Y99">
+        <v>1.08142499</v>
+      </c>
+      <c r="Z99">
+        <v>1.667E-05</v>
+      </c>
+      <c r="AA99">
+        <v>-3.889E-05</v>
+      </c>
+      <c r="AB99">
+        <v>-16.13333333</v>
+      </c>
+      <c r="AC99">
+        <v>-4.91733333</v>
+      </c>
+      <c r="AD99" t="s">
+        <v>539</v>
+      </c>
+      <c r="AE99">
+        <v>-0.1</v>
+      </c>
+      <c r="AF99">
+        <v>-28.094671</v>
+      </c>
+      <c r="AG99">
+        <v>0.015411</v>
+      </c>
+      <c r="AH99">
+        <v>17.216124</v>
+      </c>
+      <c r="AI99">
+        <v>0.07646500000000001</v>
+      </c>
+      <c r="AJ99">
+        <v>0.694775</v>
+      </c>
+      <c r="AK99">
+        <v>-1.509331</v>
+      </c>
+      <c r="AL99">
+        <v>-9.321662</v>
+      </c>
+      <c r="AM99">
+        <v>-0.030478</v>
+      </c>
+      <c r="AN99">
+        <v>-8.563257</v>
+      </c>
+      <c r="AO99">
+        <v>0.004697</v>
+      </c>
+      <c r="AP99">
+        <v>5.247478</v>
+      </c>
+      <c r="AQ99">
+        <v>0.023307</v>
+      </c>
+      <c r="AR99">
+        <v>0.6947950000000001</v>
+      </c>
+      <c r="AS99">
+        <v>-1.509203</v>
+      </c>
+      <c r="AT99">
+        <v>-2.841231</v>
+      </c>
+    </row>
+    <row r="100" spans="1:46">
+      <c r="A100" t="s">
+        <v>37</v>
+      </c>
+      <c r="B100" t="s">
+        <v>92</v>
+      </c>
+      <c r="C100" s="2">
+        <v>45969.39708081019</v>
+      </c>
+      <c r="D100" s="2">
+        <v>45969.39704861111</v>
+      </c>
+      <c r="E100">
+        <v>4206</v>
+      </c>
+      <c r="F100">
+        <v>1281.99</v>
+      </c>
+      <c r="G100">
+        <v>-33.3</v>
+      </c>
+      <c r="H100">
+        <v>3300</v>
+      </c>
+      <c r="I100" t="s">
+        <v>340</v>
+      </c>
+      <c r="J100" t="s">
+        <v>439</v>
+      </c>
+      <c r="K100" t="s">
+        <v>538</v>
+      </c>
+      <c r="L100">
+        <v>170</v>
+      </c>
+      <c r="M100">
+        <v>0</v>
+      </c>
+      <c r="N100">
+        <v>0</v>
+      </c>
+      <c r="O100">
+        <v>39.4126666667</v>
+      </c>
+      <c r="P100">
+        <v>-102.4765</v>
+      </c>
+      <c r="Q100">
+        <v>101.7</v>
+      </c>
+      <c r="R100">
+        <v>163.66</v>
+      </c>
+      <c r="S100">
+        <v>56.84</v>
+      </c>
+      <c r="T100">
+        <v>13.8</v>
+      </c>
+      <c r="U100">
+        <v>286.95</v>
+      </c>
+      <c r="V100">
+        <v>87620</v>
+      </c>
+      <c r="W100">
+        <v>0.86</v>
+      </c>
+      <c r="X100">
+        <v>0.00206402</v>
+      </c>
+      <c r="Y100">
+        <v>1.06374974</v>
+      </c>
+      <c r="Z100">
+        <v>9.3E-07</v>
+      </c>
+      <c r="AA100">
+        <v>-1.85E-06</v>
+      </c>
+      <c r="AB100">
+        <v>-0.5555555599999999</v>
+      </c>
+      <c r="AC100">
+        <v>-0.16933333</v>
+      </c>
+      <c r="AD100" t="s">
+        <v>539</v>
+      </c>
+      <c r="AE100">
+        <v>0.021636</v>
+      </c>
+      <c r="AF100">
+        <v>-27.816498</v>
+      </c>
+      <c r="AG100">
+        <v>0.015475</v>
+      </c>
+      <c r="AH100">
+        <v>17.350248</v>
+      </c>
+      <c r="AI100">
+        <v>0.076073</v>
+      </c>
+      <c r="AJ100">
+        <v>1.571213</v>
+      </c>
+      <c r="AK100">
+        <v>0.080988</v>
+      </c>
+      <c r="AL100">
+        <v>-5.124269</v>
+      </c>
+      <c r="AM100">
+        <v>0.006594</v>
+      </c>
+      <c r="AN100">
+        <v>-8.47847</v>
+      </c>
+      <c r="AO100">
+        <v>0.004717</v>
+      </c>
+      <c r="AP100">
+        <v>5.288359</v>
+      </c>
+      <c r="AQ100">
+        <v>0.023188</v>
+      </c>
+      <c r="AR100">
+        <v>1.571213</v>
+      </c>
+      <c r="AS100">
+        <v>0.08094700000000001</v>
+      </c>
+      <c r="AT100">
+        <v>-1.561847</v>
       </c>
     </row>
   </sheetData>

</xml_diff>